<commit_message>
feat: add Project column to sample-tasks.xlsx
Assigns tasks to three projects (Platform Reboot, Auth Service,
Frontend Portal) to match the now-required Project field.
</commit_message>
<xml_diff>
--- a/public/sample-tasks.xlsx
+++ b/public/sample-tasks.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:O11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,39 +407,42 @@
         <v>Task Name</v>
       </c>
       <c r="C1" t="str">
+        <v>Project</v>
+      </c>
+      <c r="D1" t="str">
         <v>Task Description</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Assignee</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Status</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Start Date</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>End Date</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Actual Start Date</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Actual End Date</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>On Hold Date</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>On Hold Reason</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Blocked By</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Dependency</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -451,29 +454,29 @@
         <v>Design system architecture</v>
       </c>
       <c r="C2" t="str">
+        <v>Platform Reboot</v>
+      </c>
+      <c r="D2" t="str">
         <v>Create high-level design for the new microservices architecture</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Alice</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Done</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>2026-06-05</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>2026-06-04</v>
       </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
       <c r="K2" t="str">
         <v/>
       </c>
@@ -484,6 +487,9 @@
         <v/>
       </c>
       <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
         <v>Completed one day early</v>
       </c>
     </row>
@@ -495,29 +501,29 @@
         <v>Set up CI/CD pipeline</v>
       </c>
       <c r="C3" t="str">
+        <v>Platform Reboot</v>
+      </c>
+      <c r="D3" t="str">
         <v>Configure GitHub Actions for automated testing and deployment</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Bob</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Done</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>2026-06-03</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>2026-06-07</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>2026-06-03</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>2026-06-07</v>
       </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
       <c r="K3" t="str">
         <v/>
       </c>
@@ -525,9 +531,12 @@
         <v/>
       </c>
       <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
         <v>T1</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
         <v/>
       </c>
     </row>
@@ -539,26 +548,26 @@
         <v>Implement user authentication</v>
       </c>
       <c r="C4" t="str">
+        <v>Auth Service</v>
+      </c>
+      <c r="D4" t="str">
         <v>Build OAuth2 login flow with JWT session tokens</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Alice</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>In Progress</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>2026-06-08</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>2026-06-14</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>2026-06-09</v>
       </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
       <c r="J4" t="str">
         <v/>
       </c>
@@ -569,9 +578,12 @@
         <v/>
       </c>
       <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
         <v>T1</v>
       </c>
-      <c r="N4" t="str">
+      <c r="O4" t="str">
         <v>Started a day late due to onboarding</v>
       </c>
     </row>
@@ -583,39 +595,42 @@
         <v>Database schema migration</v>
       </c>
       <c r="C5" t="str">
+        <v>Auth Service</v>
+      </c>
+      <c r="D5" t="str">
         <v>Write and test migration scripts for the new schema</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>Carol</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <v>On Hold</v>
       </c>
-      <c r="F5" t="str">
+      <c r="G5" t="str">
         <v>2026-06-08</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>2026-06-12</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>2026-06-08</v>
       </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
       <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v>2026-06-10</v>
       </c>
-      <c r="K5" t="str">
+      <c r="L5" t="str">
         <v>Waiting for DBA approval on table structure changes</v>
       </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
       <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
         <v>T1</v>
       </c>
-      <c r="N5" t="str">
+      <c r="O5" t="str">
         <v/>
       </c>
     </row>
@@ -627,39 +642,42 @@
         <v>Build REST API endpoints</v>
       </c>
       <c r="C6" t="str">
+        <v>Platform Reboot</v>
+      </c>
+      <c r="D6" t="str">
         <v>Implement CRUD endpoints for users, tasks, and projects</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Bob</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <v>On Hold</v>
       </c>
-      <c r="F6" t="str">
+      <c r="G6" t="str">
         <v>2026-06-10</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>2026-06-18</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>2026-06-10</v>
       </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
       <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
         <v>2026-06-13</v>
       </c>
-      <c r="K6" t="str">
+      <c r="L6" t="str">
         <v>Blocked by T4 — schema not finalised yet</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
         <v>T4</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>T3</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v/>
       </c>
     </row>
@@ -671,26 +689,26 @@
         <v>Write unit tests for auth module</v>
       </c>
       <c r="C7" t="str">
+        <v>Auth Service</v>
+      </c>
+      <c r="D7" t="str">
         <v>Achieve 80% coverage for the authentication module</v>
       </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <v>Dave</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <v>In Progress</v>
       </c>
-      <c r="F7" t="str">
+      <c r="G7" t="str">
         <v>2026-06-12</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>2026-06-16</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>2026-06-12</v>
       </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
       <c r="J7" t="str">
         <v/>
       </c>
@@ -701,9 +719,12 @@
         <v/>
       </c>
       <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
         <v>T3</v>
       </c>
-      <c r="N7" t="str">
+      <c r="O7" t="str">
         <v/>
       </c>
     </row>
@@ -715,23 +736,23 @@
         <v>Front-end integration</v>
       </c>
       <c r="C8" t="str">
+        <v>Frontend Portal</v>
+      </c>
+      <c r="D8" t="str">
         <v>Connect React app to the new backend APIs</v>
       </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <v>Alice</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <v>Todo</v>
       </c>
-      <c r="F8" t="str">
+      <c r="G8" t="str">
         <v>2026-06-17</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>2026-06-21</v>
       </c>
-      <c r="H8" t="str">
-        <v/>
-      </c>
       <c r="I8" t="str">
         <v/>
       </c>
@@ -745,9 +766,12 @@
         <v/>
       </c>
       <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
         <v>T5</v>
       </c>
-      <c r="N8" t="str">
+      <c r="O8" t="str">
         <v/>
       </c>
     </row>
@@ -759,23 +783,23 @@
         <v>Performance testing</v>
       </c>
       <c r="C9" t="str">
+        <v>Platform Reboot</v>
+      </c>
+      <c r="D9" t="str">
         <v>Load-test the API with k6, target 1000 req/s at p99 &lt; 200ms</v>
       </c>
-      <c r="D9" t="str">
+      <c r="E9" t="str">
         <v>Carol</v>
       </c>
-      <c r="E9" t="str">
+      <c r="F9" t="str">
         <v>Todo</v>
       </c>
-      <c r="F9" t="str">
+      <c r="G9" t="str">
         <v>2026-06-20</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>2026-06-24</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
       <c r="I9" t="str">
         <v/>
       </c>
@@ -786,12 +810,15 @@
         <v/>
       </c>
       <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
         <v>T5</v>
       </c>
-      <c r="M9" t="str">
+      <c r="N9" t="str">
         <v>T5,T6</v>
       </c>
-      <c r="N9" t="str">
+      <c r="O9" t="str">
         <v/>
       </c>
     </row>
@@ -803,23 +830,23 @@
         <v>Documentation</v>
       </c>
       <c r="C10" t="str">
+        <v>Platform Reboot</v>
+      </c>
+      <c r="D10" t="str">
         <v>Write API docs in OpenAPI 3.1 and update the developer wiki</v>
       </c>
-      <c r="D10" t="str">
+      <c r="E10" t="str">
         <v>Dave</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
         <v>Todo</v>
       </c>
-      <c r="F10" t="str">
+      <c r="G10" t="str">
         <v>2026-06-21</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>2026-06-25</v>
       </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
       <c r="I10" t="str">
         <v/>
       </c>
@@ -833,9 +860,12 @@
         <v/>
       </c>
       <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
         <v>T5</v>
       </c>
-      <c r="N10" t="str">
+      <c r="O10" t="str">
         <v/>
       </c>
     </row>
@@ -847,23 +877,23 @@
         <v>Production deployment</v>
       </c>
       <c r="C11" t="str">
+        <v>Platform Reboot</v>
+      </c>
+      <c r="D11" t="str">
         <v>Deploy all services to production and run smoke tests</v>
       </c>
-      <c r="D11" t="str">
+      <c r="E11" t="str">
         <v>Bob</v>
       </c>
-      <c r="E11" t="str">
+      <c r="F11" t="str">
         <v>Todo</v>
       </c>
-      <c r="F11" t="str">
+      <c r="G11" t="str">
         <v>2026-06-25</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>2026-06-27</v>
       </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
       <c r="I11" t="str">
         <v/>
       </c>
@@ -877,15 +907,18 @@
         <v/>
       </c>
       <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
         <v>T7,T8,T9</v>
       </c>
-      <c r="N11" t="str">
+      <c r="O11" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: rename Start Date / End Date to Target Start Date / Target End Date
Updates Excel column names across parser, exporter, UI labels, How to Use
guide, filter bar, tests, and sample file.
</commit_message>
<xml_diff>
--- a/public/sample-tasks.xlsx
+++ b/public/sample-tasks.xlsx
@@ -419,10 +419,10 @@
         <v>Status</v>
       </c>
       <c r="G1" t="str">
-        <v>Start Date</v>
+        <v>Target Start Date</v>
       </c>
       <c r="H1" t="str">
-        <v>End Date</v>
+        <v>Target End Date</v>
       </c>
       <c r="I1" t="str">
         <v>Actual Start Date</v>

</xml_diff>

<commit_message>
feat: add Story Points, sample download link, burndown fix, and How to Use updates
- Add Story Points column to Excel format and sample-tasks.xlsx (10 tasks, 45 SP total)
- Add Dependency column to Excel format; update REQUIRED_COLUMNS and REQUIRED_FIELDS in page.tsx
- Fix sprint burndown: cap Remaining/SP Remaining lines at today so they don't project flat into the future
- Add "Download sample file" button to How to Use section (links to /sample-tasks.xlsx)
- Rewrite How to Use guide: full 16-column table with required markers, new Explore Reports step listing all 6 sub-tabs, updated wording throughout
- Update CLAUDE.md Excel format table to reflect all current columns and auto-set date fields
- Add deployment test report (test-results/deployment-test-report.md) — 11/12 pass on prod
</commit_message>
<xml_diff>
--- a/public/sample-tasks.xlsx
+++ b/public/sample-tasks.xlsx
@@ -397,7 +397,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:P11"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="12.83203125" customWidth="1"/>
+    <col min="13" max="13" width="45.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="40.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,33 +434,36 @@
         <v>Assignee</v>
       </c>
       <c r="F1" t="str">
+        <v>Story Points</v>
+      </c>
+      <c r="G1" t="str">
         <v>Status</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Target Start Date</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Target End Date</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Actual Start Date</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Actual End Date</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>On Hold Date</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>On Hold Reason</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Blocked By</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Dependency</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -462,24 +483,24 @@
       <c r="E2" t="str">
         <v>Alice</v>
       </c>
-      <c r="F2" t="str">
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2" t="str">
         <v>Done</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>2026-06-05</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>2026-06-01</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>2026-06-04</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
       <c r="L2" t="str">
         <v/>
       </c>
@@ -490,6 +511,9 @@
         <v/>
       </c>
       <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
         <v>Completed one day early</v>
       </c>
     </row>
@@ -509,24 +533,24 @@
       <c r="E3" t="str">
         <v>Bob</v>
       </c>
-      <c r="F3" t="str">
+      <c r="F3">
+        <v>3</v>
+      </c>
+      <c r="G3" t="str">
         <v>Done</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>2026-06-03</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>2026-06-07</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>2026-06-03</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>2026-06-07</v>
       </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
       <c r="L3" t="str">
         <v/>
       </c>
@@ -534,9 +558,12 @@
         <v/>
       </c>
       <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
         <v>T1</v>
       </c>
-      <c r="O3" t="str">
+      <c r="P3" t="str">
         <v/>
       </c>
     </row>
@@ -556,21 +583,21 @@
       <c r="E4" t="str">
         <v>Alice</v>
       </c>
-      <c r="F4" t="str">
+      <c r="F4">
+        <v>8</v>
+      </c>
+      <c r="G4" t="str">
         <v>In Progress</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>2026-06-08</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>2026-06-14</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>2026-06-09</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
       <c r="K4" t="str">
         <v/>
       </c>
@@ -581,9 +608,12 @@
         <v/>
       </c>
       <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
         <v>T1</v>
       </c>
-      <c r="O4" t="str">
+      <c r="P4" t="str">
         <v>Started a day late due to onboarding</v>
       </c>
     </row>
@@ -603,34 +633,37 @@
       <c r="E5" t="str">
         <v>Carol</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5" t="str">
         <v>On Hold</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>2026-06-08</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>2026-06-12</v>
       </c>
-      <c r="I5" t="str">
+      <c r="J5" t="str">
         <v>2026-06-08</v>
       </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
       <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
         <v>2026-06-10</v>
       </c>
-      <c r="L5" t="str">
+      <c r="M5" t="str">
         <v>Waiting for DBA approval on table structure changes</v>
       </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
       <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
         <v>T1</v>
       </c>
-      <c r="O5" t="str">
+      <c r="P5" t="str">
         <v/>
       </c>
     </row>
@@ -650,34 +683,37 @@
       <c r="E6" t="str">
         <v>Bob</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="G6" t="str">
         <v>On Hold</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>2026-06-10</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>2026-06-18</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>2026-06-10</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
       <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
         <v>2026-06-13</v>
       </c>
-      <c r="L6" t="str">
+      <c r="M6" t="str">
         <v>Blocked by T4 — schema not finalised yet</v>
       </c>
-      <c r="M6" t="str">
+      <c r="N6" t="str">
         <v>T4</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>T3</v>
       </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
         <v/>
       </c>
     </row>
@@ -697,21 +733,21 @@
       <c r="E7" t="str">
         <v>Dave</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="G7" t="str">
         <v>In Progress</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>2026-06-12</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>2026-06-16</v>
       </c>
-      <c r="I7" t="str">
+      <c r="J7" t="str">
         <v>2026-06-12</v>
       </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
       <c r="K7" t="str">
         <v/>
       </c>
@@ -722,9 +758,12 @@
         <v/>
       </c>
       <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
         <v>T3</v>
       </c>
-      <c r="O7" t="str">
+      <c r="P7" t="str">
         <v/>
       </c>
     </row>
@@ -744,18 +783,18 @@
       <c r="E8" t="str">
         <v>Alice</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F8">
+        <v>5</v>
+      </c>
+      <c r="G8" t="str">
         <v>Todo</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>2026-06-17</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>2026-06-21</v>
       </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
       <c r="J8" t="str">
         <v/>
       </c>
@@ -769,9 +808,12 @@
         <v/>
       </c>
       <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
         <v>T5</v>
       </c>
-      <c r="O8" t="str">
+      <c r="P8" t="str">
         <v/>
       </c>
     </row>
@@ -791,18 +833,18 @@
       <c r="E9" t="str">
         <v>Carol</v>
       </c>
-      <c r="F9" t="str">
+      <c r="F9">
+        <v>3</v>
+      </c>
+      <c r="G9" t="str">
         <v>Todo</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>2026-06-20</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>2026-06-24</v>
       </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
       <c r="J9" t="str">
         <v/>
       </c>
@@ -813,12 +855,15 @@
         <v/>
       </c>
       <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
         <v>T5</v>
       </c>
-      <c r="N9" t="str">
+      <c r="O9" t="str">
         <v>T5,T6</v>
       </c>
-      <c r="O9" t="str">
+      <c r="P9" t="str">
         <v/>
       </c>
     </row>
@@ -838,18 +883,18 @@
       <c r="E10" t="str">
         <v>Dave</v>
       </c>
-      <c r="F10" t="str">
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" t="str">
         <v>Todo</v>
       </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>2026-06-21</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>2026-06-25</v>
       </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
       <c r="J10" t="str">
         <v/>
       </c>
@@ -863,9 +908,12 @@
         <v/>
       </c>
       <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
         <v>T5</v>
       </c>
-      <c r="O10" t="str">
+      <c r="P10" t="str">
         <v/>
       </c>
     </row>
@@ -885,18 +933,18 @@
       <c r="E11" t="str">
         <v>Bob</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F11">
+        <v>3</v>
+      </c>
+      <c r="G11" t="str">
         <v>Todo</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>2026-06-25</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>2026-06-27</v>
       </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
       <c r="J11" t="str">
         <v/>
       </c>
@@ -910,15 +958,18 @@
         <v/>
       </c>
       <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
         <v>T7,T8,T9</v>
       </c>
-      <c r="O11" t="str">
+      <c r="P11" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Validation & Testing column, on-hold history badge, and status transition logic
- Add 'Validation & Testing' as a new Kanban status between In Progress and On Hold
- Only In Progress cards can move to Validation & Testing; On Hold accepts from both
- Extract applyStatusTransition() to lib/taskUtils.ts for pure, testable status logic
- On Hold resume: set onHoldEndDate (today − 1) and preserve onHoldDate/onHoldReason
  so TaskCard can show 'Was on Hold from X to Y' badge after resuming
- Re-entering On Hold resets onHoldEndDate for a clean new hold period
- Add onHoldEndDate field to Task type, Excel parser, exporter, and sample file
- Update ChartsView, WorkloadReport, SprintReport, ReportsTabs filter with V&T status
- Update HowToUse, page.tsx, and CLAUDE.md to document all five statuses
- 36 tests passing
</commit_message>
<xml_diff>
--- a/public/sample-tasks.xlsx
+++ b/public/sample-tasks.xlsx
@@ -397,24 +397,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:Q12"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="4" max="4" width="52.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
     <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="45.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="40.83203125" customWidth="1"/>
     <col min="15" max="15" width="14.83203125" customWidth="1"/>
-    <col min="16" max="16" width="40.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="36.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,15 +456,18 @@
         <v>On Hold Date</v>
       </c>
       <c r="M1" t="str">
+        <v>On Hold End Date</v>
+      </c>
+      <c r="N1" t="str">
         <v>On Hold Reason</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Blocked By</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Dependency</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Notes</v>
       </c>
     </row>
@@ -514,6 +518,9 @@
         <v/>
       </c>
       <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
         <v>Completed one day early</v>
       </c>
     </row>
@@ -561,9 +568,12 @@
         <v/>
       </c>
       <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
         <v>T1</v>
       </c>
-      <c r="P3" t="str">
+      <c r="Q3" t="str">
         <v/>
       </c>
     </row>
@@ -587,7 +597,7 @@
         <v>8</v>
       </c>
       <c r="G4" t="str">
-        <v>In Progress</v>
+        <v>Validation &amp; Testing</v>
       </c>
       <c r="H4" t="str">
         <v>2026-06-08</v>
@@ -611,10 +621,13 @@
         <v/>
       </c>
       <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>T1</v>
       </c>
-      <c r="P4" t="str">
-        <v>Started a day late due to onboarding</v>
+      <c r="Q4" t="str">
+        <v>Implementation complete — awaiting QA sign-off</v>
       </c>
     </row>
     <row r="5">
@@ -655,15 +668,18 @@
         <v>2026-06-10</v>
       </c>
       <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
         <v>Waiting for DBA approval on table structure changes</v>
       </c>
-      <c r="N5" t="str">
-        <v/>
-      </c>
       <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
         <v>T1</v>
       </c>
-      <c r="P5" t="str">
+      <c r="Q5" t="str">
         <v/>
       </c>
     </row>
@@ -705,15 +721,18 @@
         <v>2026-06-13</v>
       </c>
       <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
         <v>Blocked by T4 — schema not finalised yet</v>
       </c>
-      <c r="N6" t="str">
+      <c r="O6" t="str">
         <v>T4</v>
       </c>
-      <c r="O6" t="str">
+      <c r="P6" t="str">
         <v>T3</v>
       </c>
-      <c r="P6" t="str">
+      <c r="Q6" t="str">
         <v/>
       </c>
     </row>
@@ -761,9 +780,12 @@
         <v/>
       </c>
       <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
         <v>T3</v>
       </c>
-      <c r="P7" t="str">
+      <c r="Q7" t="str">
         <v/>
       </c>
     </row>
@@ -772,31 +794,31 @@
         <v>T7</v>
       </c>
       <c r="B8" t="str">
-        <v>Front-end integration</v>
+        <v>API integration testing</v>
       </c>
       <c r="C8" t="str">
-        <v>Frontend Portal</v>
+        <v>Platform Reboot</v>
       </c>
       <c r="D8" t="str">
-        <v>Connect React app to the new backend APIs</v>
+        <v>End-to-end tests covering all REST endpoints and edge cases</v>
       </c>
       <c r="E8" t="str">
-        <v>Alice</v>
+        <v>Carol</v>
       </c>
       <c r="F8">
         <v>5</v>
       </c>
       <c r="G8" t="str">
-        <v>Todo</v>
+        <v>Validation &amp; Testing</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-06-17</v>
+        <v>2026-06-14</v>
       </c>
       <c r="I8" t="str">
-        <v>2026-06-21</v>
+        <v>2026-06-18</v>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>2026-06-14</v>
       </c>
       <c r="K8" t="str">
         <v/>
@@ -811,10 +833,13 @@
         <v/>
       </c>
       <c r="O8" t="str">
-        <v>T5</v>
+        <v/>
       </c>
       <c r="P8" t="str">
-        <v/>
+        <v>T2,T3</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Running regression suite against staging environment</v>
       </c>
     </row>
     <row r="9">
@@ -822,28 +847,28 @@
         <v>T8</v>
       </c>
       <c r="B9" t="str">
-        <v>Performance testing</v>
+        <v>Front-end integration</v>
       </c>
       <c r="C9" t="str">
-        <v>Platform Reboot</v>
+        <v>Frontend Portal</v>
       </c>
       <c r="D9" t="str">
-        <v>Load-test the API with k6, target 1000 req/s at p99 &lt; 200ms</v>
+        <v>Connect React app to the new backend APIs</v>
       </c>
       <c r="E9" t="str">
-        <v>Carol</v>
+        <v>Alice</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G9" t="str">
         <v>Todo</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-06-20</v>
+        <v>2026-06-19</v>
       </c>
       <c r="I9" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-23</v>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -858,12 +883,15 @@
         <v/>
       </c>
       <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
         <v>T5</v>
       </c>
-      <c r="O9" t="str">
-        <v>T5,T6</v>
-      </c>
-      <c r="P9" t="str">
+      <c r="Q9" t="str">
         <v/>
       </c>
     </row>
@@ -872,28 +900,28 @@
         <v>T9</v>
       </c>
       <c r="B10" t="str">
-        <v>Documentation</v>
+        <v>Performance testing</v>
       </c>
       <c r="C10" t="str">
         <v>Platform Reboot</v>
       </c>
       <c r="D10" t="str">
-        <v>Write API docs in OpenAPI 3.1 and update the developer wiki</v>
+        <v>Load-test the API with k6, target 1000 req/s at p99 &lt; 200ms</v>
       </c>
       <c r="E10" t="str">
-        <v>Dave</v>
+        <v>Carol</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" t="str">
         <v>Todo</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-06-21</v>
+        <v>2026-06-22</v>
       </c>
       <c r="I10" t="str">
-        <v>2026-06-25</v>
+        <v>2026-06-26</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -914,6 +942,9 @@
         <v>T5</v>
       </c>
       <c r="P10" t="str">
+        <v>T5,T6</v>
+      </c>
+      <c r="Q10" t="str">
         <v/>
       </c>
     </row>
@@ -922,25 +953,25 @@
         <v>T10</v>
       </c>
       <c r="B11" t="str">
-        <v>Production deployment</v>
+        <v>Documentation</v>
       </c>
       <c r="C11" t="str">
         <v>Platform Reboot</v>
       </c>
       <c r="D11" t="str">
-        <v>Deploy all services to production and run smoke tests</v>
+        <v>Write API docs in OpenAPI 3.1 and update the developer wiki</v>
       </c>
       <c r="E11" t="str">
-        <v>Bob</v>
+        <v>Dave</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G11" t="str">
         <v>Todo</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-06-25</v>
+        <v>2026-06-23</v>
       </c>
       <c r="I11" t="str">
         <v>2026-06-27</v>
@@ -961,15 +992,71 @@
         <v/>
       </c>
       <c r="O11" t="str">
-        <v>T7,T8,T9</v>
+        <v/>
       </c>
       <c r="P11" t="str">
+        <v>T5</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>T11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Production deployment</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Platform Reboot</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Deploy all services to production and run smoke tests</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Bob</v>
+      </c>
+      <c r="F12">
+        <v>3</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Todo</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-06-27</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2026-06-29</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v>T8,T9,T10</v>
+      </c>
+      <c r="Q12" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>